<commit_message>
TCC: verificação independente dos modos Série e Paralelo e casos de borda
- Nova Seção 3.9.3 e 4.3.3: recálculo independente de Carnaubal–Batalhão e
  Fogareiro–Quixeramobim a partir da descrição do texto, sem importar o
  simulador; 5.280 balanços mensais, 0 divergências (Tabela 13, Código-fonte 6).
- Três casos controlados novos (transferência limitada pelo fornecedor,
  transferência com vertimento no receptor, segunda unidade sem volume no
  Paralelo), todos aprovados na versão de referência e na atual.
- Conclusão restringida às configurações verificadas; resumo e abstract
  atualizados; script e planilha de casos no material complementar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BYniudVLYZZcBkfNP72QEN
</commit_message>
<xml_diff>
--- a/tcc/material_complementar/05_casos_controlados_e_sensibilidade/casos_controlados.xlsx
+++ b/tcc/material_complementar/05_casos_controlados_e_sensibilidade/casos_controlados.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -686,6 +686,87 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Transferência limitada pelo fornecedor (Série)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Receptor: 10 hm³, V0 = 20%, gatilho 30%; fornecedor: 50 hm³, V0 = 0,1 hm³; T = 100 L/s (0,2592 hm³/mês)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>T = 0,1000 hm³ no mês 1 e 0 no mês 2; fornecedor com V = 0; receptor com V = 2,1000 hm³</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>T = 0.1000; 0.0000 hm³; V fornecedor = 0.0000; V receptor = 2.1000 hm³</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Transferência com vertimento no receptor (Série)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Receptor: 1 hm³, V0 = 20%, gatilho 30%; fornecedor: 50 hm³, V0 = 40 hm³; T = 1 m³/s (2,592 hm³/mês)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>mês 1: T = 2,592 hm³, receptor cheio (1,000 hm³) e S = 1,792 hm³; fornecedor com 37,408 hm³; mês 2 sem transferência</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>T = 2.592; 0.000 hm³; V receptor = 1.000; S = 1.792; V fornecedor = 37.408 hm³</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Segunda unidade sem volume (Paralelo)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>R1: 10 hm³, V0 = 0,3 hm³ (3%), gatilho 20%; R2: 10 hm³, V0 = 0,1 hm³; Dconj = 100 L/s (0,2592 hm³/mês)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>R1 permanece responsável: R = 0,2592; 0,0408; 0 hm³, com falha nos meses 2 e 3; R2 sem retirada e com V = 0,1 hm³</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>R1 = 0.2592; 0.0408; 0.0000 hm³; falhas R1 = ['Não', 'Sim', 'Sim']; R2 retirada = 0.0000; V R2 = 0.1000 hm³</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>